<commit_message>
feat(ai): categorize 16 domain discovery cate words by perception objects
</commit_message>
<xml_diff>
--- a/data/analyze/final_16_domain_discovery_words.xlsx
+++ b/data/analyze/final_16_domain_discovery_words.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="53">
   <si>
     <t>word</t>
   </si>
@@ -37,6 +37,12 @@
     <t>domain_category</t>
   </si>
   <si>
+    <t>perception_object</t>
+  </si>
+  <si>
+    <t>target_description</t>
+  </si>
+  <si>
     <t>spectacular</t>
   </si>
   <si>
@@ -155,6 +161,18 @@
   </si>
   <si>
     <t>Flight Motion &amp; Somatic State (飞行体感与生理反应)</t>
+  </si>
+  <si>
+    <t>1. 高空自然景观与美学震撼 (Aerial Scenery &amp; Visual Nature)</t>
+  </si>
+  <si>
+    <t>2. 飞行体感与机舱躯体反应 (Aircraft Riding &amp; Flight Motion)</t>
+  </si>
+  <si>
+    <t>俯瞰雪山峡谷、高空视觉奇观、极致壮观美感</t>
+  </si>
+  <si>
+    <t>机舱颠簸感、晕机反应、密闭空间压抑焦虑</t>
   </si>
 </sst>
 </file>
@@ -512,10 +530,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,373 +555,475 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>1616</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>1612</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>304</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>276</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C9">
         <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H12" t="s">
+        <v>49</v>
+      </c>
+      <c r="I12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>48</v>
+      </c>
+      <c r="H13" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G14" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C16">
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>48</v>
+      </c>
+      <c r="H16" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="H17" t="s">
+        <v>49</v>
+      </c>
+      <c r="I17" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): categorize 16 cate words into 3 perception target categories
</commit_message>
<xml_diff>
--- a/data/analyze/final_16_domain_discovery_words.xlsx
+++ b/data/analyze/final_16_domain_discovery_words.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="57">
   <si>
     <t>word</t>
   </si>
@@ -43,6 +43,9 @@
     <t>target_description</t>
   </si>
   <si>
+    <t>perception_object_3_classes</t>
+  </si>
+  <si>
     <t>spectacular</t>
   </si>
   <si>
@@ -173,6 +176,15 @@
   </si>
   <si>
     <t>机舱颠簸感、晕机反应、密闭空间压抑焦虑</t>
+  </si>
+  <si>
+    <t>1. 高空自然景观美学震撼 (Aerial Visual Scenery &amp; Aesthetics)</t>
+  </si>
+  <si>
+    <t>3. 总体观光体验极致赞赏 (Overall Tour Excellence &amp; Appraisal)</t>
+  </si>
+  <si>
+    <t>2. 机舱乘坐体感与生理反应 (Aircraft Motion &amp; Physical Distress)</t>
   </si>
 </sst>
 </file>
@@ -530,10 +542,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -561,469 +573,520 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>1616</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>1612</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>304</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>276</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8">
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>53</v>
+      </c>
+      <c r="J10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>53</v>
+      </c>
+      <c r="J13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>52</v>
+      </c>
+      <c r="J15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16">
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>53</v>
+      </c>
+      <c r="J16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I17" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="J17" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): categorize 16 cate words by self vs environment perception entities
</commit_message>
<xml_diff>
--- a/data/analyze/final_16_domain_discovery_words.xlsx
+++ b/data/analyze/final_16_domain_discovery_words.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="65">
   <si>
     <t>word</t>
   </si>
@@ -46,6 +46,12 @@
     <t>perception_object_3_classes</t>
   </si>
   <si>
+    <t>perceptual_entity</t>
+  </si>
+  <si>
+    <t>entity_explanation</t>
+  </si>
+  <si>
     <t>spectacular</t>
   </si>
   <si>
@@ -185,6 +191,24 @@
   </si>
   <si>
     <t>2. 机舱乘坐体感与生理反应 (Aircraft Motion &amp; Physical Distress)</t>
+  </si>
+  <si>
+    <t>2. 外部自然景观对象 (External Physical Scenery &amp; Environment)</t>
+  </si>
+  <si>
+    <t>3. 行程认知评估与主观震撼 (Cognitive Appraisal &amp; Experience Impact)</t>
+  </si>
+  <si>
+    <t>1. 自我躯体与内感感知 (Self / Somatic Internal Perception)</t>
+  </si>
+  <si>
+    <t>感知对象为外部物理景色（雪山、峡谷、海洋等高空自然风光）</t>
+  </si>
+  <si>
+    <t>感知对象为整趟行程的心理震撼与认知评价（敬畏、现象级超预期）</t>
+  </si>
+  <si>
+    <t>感知主体为游客自身（身体晕眩、密闭空间恐惧等躯体与生理反应）</t>
   </si>
 </sst>
 </file>
@@ -542,10 +566,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -576,517 +600,619 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>1616</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K2" t="s">
+        <v>59</v>
+      </c>
+      <c r="L2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>1612</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>57</v>
+      </c>
+      <c r="K3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>304</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K5" t="s">
+        <v>60</v>
+      </c>
+      <c r="L5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>276</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>57</v>
+      </c>
+      <c r="K7" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K8" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C9">
         <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K9" t="s">
+        <v>59</v>
+      </c>
+      <c r="L9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10">
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>58</v>
+      </c>
+      <c r="K10" t="s">
+        <v>61</v>
+      </c>
+      <c r="L10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C11">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C12">
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J12" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K12" t="s">
+        <v>59</v>
+      </c>
+      <c r="L12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I13" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+        <v>58</v>
+      </c>
+      <c r="K13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I14" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K14" t="s">
+        <v>60</v>
+      </c>
+      <c r="L14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>56</v>
+      </c>
+      <c r="K15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C16">
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H16" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>58</v>
+      </c>
+      <c r="K16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J17" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="K17" t="s">
+        <v>59</v>
+      </c>
+      <c r="L17" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): enrich 16 cate words with emotions polarities and real review context sentences
</commit_message>
<xml_diff>
--- a/data/analyze/final_16_domain_discovery_words.xlsx
+++ b/data/analyze/final_16_domain_discovery_words.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="102">
   <si>
     <t>word</t>
   </si>
@@ -52,6 +52,15 @@
     <t>entity_explanation</t>
   </si>
   <si>
+    <t>emotion_category</t>
+  </si>
+  <si>
+    <t>polarity</t>
+  </si>
+  <si>
+    <t>context_sentence_example</t>
+  </si>
+  <si>
     <t>spectacular</t>
   </si>
   <si>
@@ -209,6 +218,108 @@
   </si>
   <si>
     <t>感知主体为游客自身（身体晕眩、密闭空间恐惧等躯体与生理反应）</t>
+  </si>
+  <si>
+    <t>Awe / Joy (高空视觉震撼与喜悦)</t>
+  </si>
+  <si>
+    <t>Awe / Delight (认知震撼与惊叹)</t>
+  </si>
+  <si>
+    <t>Joy / Serenity (宜人赏心悦目)</t>
+  </si>
+  <si>
+    <t>Awe / Wonder (敬畏与震慑)</t>
+  </si>
+  <si>
+    <t>Trust / Joy (极度赞赏与信任)</t>
+  </si>
+  <si>
+    <t>Awe / Joy (现象级震撼与赞叹)</t>
+  </si>
+  <si>
+    <t>Awe / Reverence (雄伟壮丽与崇高感)</t>
+  </si>
+  <si>
+    <t>Surprise / Wonder (超现实梦幻与惊奇)</t>
+  </si>
+  <si>
+    <t>Disgust / Physical Distress (躯体晕眩与不适)</t>
+  </si>
+  <si>
+    <t>Awe / Excitement (屏息震撼地)</t>
+  </si>
+  <si>
+    <t>Awe / Fascination (目眩神迷致敬)</t>
+  </si>
+  <si>
+    <t>Fear / Anxiety (密闭空间焦虑与恐惧)</t>
+  </si>
+  <si>
+    <t>Awe / Reverence (敬畏肃然感)</t>
+  </si>
+  <si>
+    <t>Awe / Surprise (目眩震撼地)</t>
+  </si>
+  <si>
+    <t>Fear / Panic (密闭恐惧发作)</t>
+  </si>
+  <si>
+    <t>Awe / Aesthetics (崇高极致美感)</t>
+  </si>
+  <si>
+    <t>Positive (正向)</t>
+  </si>
+  <si>
+    <t>Negative (负向)</t>
+  </si>
+  <si>
+    <t>The aerial view of the canyon was absolute spectacular.</t>
+  </si>
+  <si>
+    <t>An incredible helicopter experience over the glaciers.</t>
+  </si>
+  <si>
+    <t>Smooth scenic flight with crystal clear views.</t>
+  </si>
+  <si>
+    <t>We stood in silent awe watching the peak from the air.</t>
+  </si>
+  <si>
+    <t>Our pilot provided an exceptional guided commentary.</t>
+  </si>
+  <si>
+    <t>The pilot's flying skills were simply phenomenal.</t>
+  </si>
+  <si>
+    <t>Floating past the majestic mountain range was dreamlike.</t>
+  </si>
+  <si>
+    <t>Hovering above the clouds felt completely surreal.</t>
+  </si>
+  <si>
+    <t>The turbulence made several passengers feel airsick.</t>
+  </si>
+  <si>
+    <t>The helicopter turned into the valley breathtakingly.</t>
+  </si>
+  <si>
+    <t>The glacier ice patterns were utterly mesmerizing.</t>
+  </si>
+  <si>
+    <t>The tiny seating area made me feel claustrophobic.</t>
+  </si>
+  <si>
+    <t>I was left awed by the sheer scale of the landscape.</t>
+  </si>
+  <si>
+    <t>The sun illuminated the cliff edge stunningly.</t>
+  </si>
+  <si>
+    <t>My claustrophobia kicked in during the doorless ride.</t>
+  </si>
+  <si>
+    <t>A sublime combination of aerial freedom and beauty.</t>
   </si>
 </sst>
 </file>
@@ -566,10 +677,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -606,613 +717,766 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2">
         <v>1616</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M2" t="s">
+        <v>68</v>
+      </c>
+      <c r="N2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3">
         <v>1612</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M3" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M4" t="s">
+        <v>70</v>
+      </c>
+      <c r="N4" t="s">
+        <v>84</v>
+      </c>
+      <c r="O4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>304</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M5" t="s">
+        <v>71</v>
+      </c>
+      <c r="N5" t="s">
+        <v>84</v>
+      </c>
+      <c r="O5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>276</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M6" t="s">
+        <v>72</v>
+      </c>
+      <c r="N6" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M7" t="s">
+        <v>73</v>
+      </c>
+      <c r="N7" t="s">
+        <v>84</v>
+      </c>
+      <c r="O7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M8" t="s">
+        <v>74</v>
+      </c>
+      <c r="N8" t="s">
+        <v>84</v>
+      </c>
+      <c r="O8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C9">
         <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M9" t="s">
+        <v>75</v>
+      </c>
+      <c r="N9" t="s">
+        <v>84</v>
+      </c>
+      <c r="O9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="K10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>67</v>
+      </c>
+      <c r="M10" t="s">
+        <v>76</v>
+      </c>
+      <c r="N10" t="s">
+        <v>85</v>
+      </c>
+      <c r="O10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C11">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I11" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" t="s">
+        <v>84</v>
+      </c>
+      <c r="O11" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C12">
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G12" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J12" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L12" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M12" t="s">
+        <v>78</v>
+      </c>
+      <c r="N12" t="s">
+        <v>84</v>
+      </c>
+      <c r="O12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J13" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="K13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>67</v>
+      </c>
+      <c r="M13" t="s">
+        <v>79</v>
+      </c>
+      <c r="N13" t="s">
+        <v>85</v>
+      </c>
+      <c r="O13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M14" t="s">
+        <v>80</v>
+      </c>
+      <c r="N14" t="s">
+        <v>84</v>
+      </c>
+      <c r="O14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I15" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J15" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L15" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+        <v>65</v>
+      </c>
+      <c r="M15" t="s">
+        <v>81</v>
+      </c>
+      <c r="N15" t="s">
+        <v>84</v>
+      </c>
+      <c r="O15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C16">
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E16" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G16" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H16" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J16" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="K16" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>67</v>
+      </c>
+      <c r="M16" t="s">
+        <v>82</v>
+      </c>
+      <c r="N16" t="s">
+        <v>85</v>
+      </c>
+      <c r="O16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F17" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I17" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K17" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L17" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+      <c r="M17" t="s">
+        <v>83</v>
+      </c>
+      <c r="N17" t="s">
+        <v>84</v>
+      </c>
+      <c r="O17" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): extract empirical sentences and star ratings for 16 domain discovery words
</commit_message>
<xml_diff>
--- a/data/analyze/final_16_domain_discovery_words.xlsx
+++ b/data/analyze/final_16_domain_discovery_words.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="123">
   <si>
     <t>word</t>
   </si>
@@ -61,6 +61,18 @@
     <t>context_sentence_example</t>
   </si>
   <si>
+    <t>empirical_mean_rating</t>
+  </si>
+  <si>
+    <t>empirical_median_rating</t>
+  </si>
+  <si>
+    <t>empirical_polarity</t>
+  </si>
+  <si>
+    <t>real_corpus_sentence_example</t>
+  </si>
+  <si>
     <t>spectacular</t>
   </si>
   <si>
@@ -320,6 +332,57 @@
   </si>
   <si>
     <t>A sublime combination of aerial freedom and beauty.</t>
+  </si>
+  <si>
+    <t>Positive (Mean Rating &gt;= 3.0)</t>
+  </si>
+  <si>
+    <t>From our communication before the tour with Lindsey to our Flight there and back with pilot Brendon and our tour on the ground with Miss Gigi this was an all around spectacular experience</t>
+  </si>
+  <si>
+    <t>It was all incredible</t>
+  </si>
+  <si>
+    <t>And then when we landed our driver took us to some of the best scenic spots on the south rim, ending with a lunch at Grand Canyon Village</t>
+  </si>
+  <si>
+    <t>Seeing the Grand Canyon from above, in all its wonder, will delight you and the learnings you will walk away with will leave you in awe</t>
+  </si>
+  <si>
+    <t>Exceptional customer service and a once in a lifetime trip</t>
+  </si>
+  <si>
+    <t>This was a phenomenal experience</t>
+  </si>
+  <si>
+    <t>It was such a magica experience , the colours of the foliage and the sighting of bears , plus Mt MacKinley looking majestic made our flight  extra special</t>
+  </si>
+  <si>
+    <t>The flight across Vancouver Island was simply amazing, the views were almost surreal</t>
+  </si>
+  <si>
+    <t>There was enough air flow in the cabin that it was not stuffy for those that may get airsick</t>
+  </si>
+  <si>
+    <t>On the other side, the tour was breathtakingly amazing</t>
+  </si>
+  <si>
+    <t>The views we saw from the flight were beautiful and mesmerizing</t>
+  </si>
+  <si>
+    <t>I am afraid of heights, get motion sickness and claustrophobic</t>
+  </si>
+  <si>
+    <t>I highly recommend going on this trip if you're looking for a new way to orient yourself with the islands and to just be awed at the beauty of Hawaii</t>
+  </si>
+  <si>
+    <t>Landing on the glacier (though I have been on many) was thrilling and stunningly beautiful - don't miss it</t>
+  </si>
+  <si>
+    <t>The planes are small, so if you have claustrophobia that might be an issue</t>
+  </si>
+  <si>
+    <t>This flight was great and the narration was really very interesting and the landing was just sublime</t>
   </si>
 </sst>
 </file>
@@ -677,10 +740,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -726,757 +789,961 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>1616</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="N2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O2" t="s">
-        <v>86</v>
+        <v>90</v>
+      </c>
+      <c r="P2">
+        <v>4.95</v>
+      </c>
+      <c r="Q2">
+        <v>5</v>
+      </c>
+      <c r="R2" t="s">
+        <v>106</v>
+      </c>
+      <c r="S2" t="s">
+        <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <v>1612</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O3" t="s">
-        <v>87</v>
+        <v>91</v>
+      </c>
+      <c r="P3">
+        <v>4.97</v>
+      </c>
+      <c r="Q3">
+        <v>5</v>
+      </c>
+      <c r="R3" t="s">
+        <v>106</v>
+      </c>
+      <c r="S3" t="s">
+        <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O4" t="s">
-        <v>88</v>
+        <v>92</v>
+      </c>
+      <c r="P4">
+        <v>4.77</v>
+      </c>
+      <c r="Q4">
+        <v>5</v>
+      </c>
+      <c r="R4" t="s">
+        <v>106</v>
+      </c>
+      <c r="S4" t="s">
+        <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C5">
         <v>304</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="N5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O5" t="s">
-        <v>89</v>
+        <v>93</v>
+      </c>
+      <c r="P5">
+        <v>4.96</v>
+      </c>
+      <c r="Q5">
+        <v>5</v>
+      </c>
+      <c r="R5" t="s">
+        <v>106</v>
+      </c>
+      <c r="S5" t="s">
+        <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>276</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="N6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O6" t="s">
-        <v>90</v>
+        <v>94</v>
+      </c>
+      <c r="P6">
+        <v>4.98</v>
+      </c>
+      <c r="Q6">
+        <v>5</v>
+      </c>
+      <c r="R6" t="s">
+        <v>106</v>
+      </c>
+      <c r="S6" t="s">
+        <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O7" t="s">
-        <v>91</v>
+        <v>95</v>
+      </c>
+      <c r="P7">
+        <v>4.97</v>
+      </c>
+      <c r="Q7">
+        <v>5</v>
+      </c>
+      <c r="R7" t="s">
+        <v>106</v>
+      </c>
+      <c r="S7" t="s">
+        <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C8">
         <v>165</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L8" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="N8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O8" t="s">
-        <v>92</v>
+        <v>96</v>
+      </c>
+      <c r="P8">
+        <v>4.97</v>
+      </c>
+      <c r="Q8">
+        <v>5</v>
+      </c>
+      <c r="R8" t="s">
+        <v>106</v>
+      </c>
+      <c r="S8" t="s">
+        <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:19">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C9">
         <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="N9" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O9" t="s">
-        <v>93</v>
+        <v>97</v>
+      </c>
+      <c r="P9">
+        <v>4.96</v>
+      </c>
+      <c r="Q9">
+        <v>5</v>
+      </c>
+      <c r="R9" t="s">
+        <v>106</v>
+      </c>
+      <c r="S9" t="s">
+        <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:19">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C10">
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="J10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="M10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="N10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O10" t="s">
-        <v>94</v>
+        <v>98</v>
+      </c>
+      <c r="P10">
+        <v>4.84</v>
+      </c>
+      <c r="Q10">
+        <v>5</v>
+      </c>
+      <c r="R10" t="s">
+        <v>106</v>
+      </c>
+      <c r="S10" t="s">
+        <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:19">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M11" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N11" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O11" t="s">
-        <v>95</v>
+        <v>99</v>
+      </c>
+      <c r="P11">
+        <v>5</v>
+      </c>
+      <c r="Q11">
+        <v>5</v>
+      </c>
+      <c r="R11" t="s">
+        <v>106</v>
+      </c>
+      <c r="S11" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:19">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C12">
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I12" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M12" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="N12" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O12" t="s">
-        <v>96</v>
+        <v>100</v>
+      </c>
+      <c r="P12">
+        <v>4.96</v>
+      </c>
+      <c r="Q12">
+        <v>5</v>
+      </c>
+      <c r="R12" t="s">
+        <v>106</v>
+      </c>
+      <c r="S12" t="s">
+        <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:19">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C13">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G13" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H13" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I13" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="J13" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="M13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="N13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O13" t="s">
-        <v>97</v>
+        <v>101</v>
+      </c>
+      <c r="P13">
+        <v>5</v>
+      </c>
+      <c r="Q13">
+        <v>5</v>
+      </c>
+      <c r="R13" t="s">
+        <v>106</v>
+      </c>
+      <c r="S13" t="s">
+        <v>118</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:19">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="L14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="N14" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O14" t="s">
-        <v>98</v>
+        <v>102</v>
+      </c>
+      <c r="P14">
+        <v>4.93</v>
+      </c>
+      <c r="Q14">
+        <v>5</v>
+      </c>
+      <c r="R14" t="s">
+        <v>106</v>
+      </c>
+      <c r="S14" t="s">
+        <v>119</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:19">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E15" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G15" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I15" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J15" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K15" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M15" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="N15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O15" t="s">
-        <v>99</v>
+        <v>103</v>
+      </c>
+      <c r="P15">
+        <v>5</v>
+      </c>
+      <c r="Q15">
+        <v>5</v>
+      </c>
+      <c r="R15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S15" t="s">
+        <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:19">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C16">
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F16" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H16" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="J16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="M16" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="N16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O16" t="s">
-        <v>100</v>
+        <v>104</v>
+      </c>
+      <c r="P16">
+        <v>5</v>
+      </c>
+      <c r="Q16">
+        <v>5</v>
+      </c>
+      <c r="R16" t="s">
+        <v>106</v>
+      </c>
+      <c r="S16" t="s">
+        <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:19">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G17" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H17" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I17" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K17" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="N17" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O17" t="s">
-        <v>101</v>
+        <v>105</v>
+      </c>
+      <c r="P17">
+        <v>5</v>
+      </c>
+      <c r="Q17">
+        <v>5</v>
+      </c>
+      <c r="R17" t="s">
+        <v>106</v>
+      </c>
+      <c r="S17" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>